<commit_message>
feat: event ECM/setup IA, module packs, notifications, and account menu
Ship Scheda tecnica L3 with registration fees, Formazione ECM faculty/griglia, anagrafiche role tabs, Starter/Pro/Intelligence/Extra modules with upgrade gates, product notifications, feedback reviews, and profile avatar menu replacing Esci.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/assets/lean-event/import/lean-event-rubrica-contatti.xlsx
+++ b/public/assets/lean-event/import/lean-event-rubrica-contatti.xlsx
@@ -447,7 +447,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:AG2"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -460,58 +460,146 @@
     <col min="9" max="9" width="22.83203125" customWidth="1"/>
     <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="22.83203125" customWidth="1"/>
+    <col min="14" max="14" width="22.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="22.83203125" customWidth="1"/>
+    <col min="21" max="21" width="22.83203125" customWidth="1"/>
+    <col min="22" max="22" width="22.83203125" customWidth="1"/>
+    <col min="23" max="23" width="22.83203125" customWidth="1"/>
+    <col min="24" max="24" width="22.83203125" customWidth="1"/>
+    <col min="25" max="25" width="22.83203125" customWidth="1"/>
+    <col min="26" max="26" width="22.83203125" customWidth="1"/>
+    <col min="27" max="27" width="22.83203125" customWidth="1"/>
+    <col min="28" max="28" width="22.83203125" customWidth="1"/>
+    <col min="29" max="29" width="22.83203125" customWidth="1"/>
+    <col min="30" max="30" width="22.83203125" customWidth="1"/>
+    <col min="31" max="31" width="22.83203125" customWidth="1"/>
+    <col min="32" max="32" width="22.83203125" customWidth="1"/>
+    <col min="33" max="33" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Vocativo</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Titolo</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Cognome</v>
+      </c>
+      <c r="D1" t="str">
         <v>Nome</v>
       </c>
-      <c r="B1" t="str">
-        <v>Cognome</v>
-      </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>Email</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
+        <v>Etichetta email</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Email 2</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Etichetta email 2</v>
+      </c>
+      <c r="I1" t="str">
         <v>Codice fiscale</v>
       </c>
-      <c r="E1" t="str">
+      <c r="J1" t="str">
         <v>Telefono</v>
       </c>
-      <c r="F1" t="str">
+      <c r="K1" t="str">
         <v>Etichetta telefono</v>
       </c>
-      <c r="G1" t="str">
+      <c r="L1" t="str">
         <v>Telefono 2</v>
       </c>
-      <c r="H1" t="str">
+      <c r="M1" t="str">
         <v>Etichetta telefono 2</v>
       </c>
-      <c r="I1" t="str">
+      <c r="N1" t="str">
+        <v>Data di nascita</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Tag</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Indirizzo</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Città</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Provincia</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Regione</v>
+      </c>
+      <c r="T1" t="str">
+        <v>CAP</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Nazione</v>
+      </c>
+      <c r="V1" t="str">
         <v>Organizzazione</v>
       </c>
-      <c r="J1" t="str">
-        <v>Tag</v>
-      </c>
-      <c r="K1" t="str">
+      <c r="W1" t="str">
+        <v>Indirizzo ente</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Città ente</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Provincia ente</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Regione ente</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>CAP ente</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Nazione ente</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Ruolo aziendale</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Preferenze alimentari</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Mobilità ridotta</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Richieste personali</v>
+      </c>
+      <c r="AG1" t="str">
         <v>Note</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Egregio</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Dottore</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Rossi</v>
+      </c>
+      <c r="D2" t="str">
         <v>Mario</v>
       </c>
-      <c r="B2" t="str">
-        <v>Rossi</v>
-      </c>
-      <c r="C2" t="str">
+      <c r="E2" t="str">
         <v>mario.rossi@esempio.it</v>
-      </c>
-      <c r="D2" t="str">
-        <v>RSSMRA80A01H501Z</v>
-      </c>
-      <c r="E2" t="str">
-        <v>+39 051 1234567</v>
       </c>
       <c r="F2" t="str">
         <v>Principale</v>
@@ -523,18 +611,84 @@
         <v/>
       </c>
       <c r="I2" t="str">
+        <v>RSSMRA80A01H501Z</v>
+      </c>
+      <c r="J2" t="str">
+        <v>+39 051 1234567</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Principale</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>01/01/1980</v>
+      </c>
+      <c r="O2" t="str">
+        <v>docente, sponsor</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Via Roma 1</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Bologna</v>
+      </c>
+      <c r="R2" t="str">
+        <v>BO</v>
+      </c>
+      <c r="S2" t="str">
+        <v>Emilia-Romagna</v>
+      </c>
+      <c r="T2" t="str">
+        <v>40121</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Italia</v>
+      </c>
+      <c r="V2" t="str">
         <v>I&amp;C srl</v>
       </c>
-      <c r="J2" t="str">
-        <v>docente, sponsor</v>
-      </c>
-      <c r="K2" t="str">
+      <c r="W2" t="str">
+        <v>Via dell'Industria 10</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Bologna</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>BO</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Emilia-Romagna</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>40127</v>
+      </c>
+      <c r="AB2" t="str">
+        <v>Italia</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Dirigente</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>Vegetariano</v>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+      <c r="AG2" t="str">
         <v>Riga di esempio — puoi eliminarla</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AG2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>